<commit_message>
Agrega proyecto Power Query: consolidacion de 3 sucursales con datos sucios
</commit_message>
<xml_diff>
--- a/INDEX-MATCH-2026..xlsx
+++ b/INDEX-MATCH-2026..xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{29A5CB5E-ECC9-4C7C-81AA-51ACAECE7430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C66D5338-ACB6-4156-A238-6DB7F508D0F7}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{29A5CB5E-ECC9-4C7C-81AA-51ACAECE7430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D04AFE1E-6E89-43D2-831D-69D8DDB0FD85}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{6A60A910-AFD6-4FAF-98E3-80B739492C98}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6A60A910-AFD6-4FAF-98E3-80B739492C98}"/>
   </bookViews>
   <sheets>
     <sheet name="Basico" sheetId="1" r:id="rId1"/>
@@ -322,10 +322,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -346,7 +346,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -643,7 +643,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0BFB423-5AAB-48D9-9681-45EE38B28788}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -891,7 +891,10 @@
       <c r="B16" s="4">
         <v>110</v>
       </c>
-      <c r="C16" s="1"/>
+      <c r="C16" s="1" t="str">
+        <f>INDEX(B4:B13, MATCH(B16,A4:A13,0))</f>
+        <v>Elena</v>
+      </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -917,7 +920,10 @@
         <f>INDEX(C4:C13,MATCH(B16,A4:A13,0))</f>
         <v>Ventas</v>
       </c>
-      <c r="C18" s="1"/>
+      <c r="C18" s="1" t="str">
+        <f>INDEX(C4:C13, MATCH(B16,A4:A13,0))</f>
+        <v>Ventas</v>
+      </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -956,7 +962,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11CA828C-9603-4E5F-BC15-E527C45831B6}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -1001,7 +1007,10 @@
         <v>Luis</v>
       </c>
       <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="D4" s="1" t="str">
+        <f>INDEX(Basico!B4:B13, MATCH(B3,Basico!A4:A13,0))</f>
+        <v>Luis</v>
+      </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1043,7 +1052,10 @@
         <v>Santo Domingo</v>
       </c>
       <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+      <c r="D7" s="1">
+        <f>INDEX(Basico!D4:D13,MATCH(B3,Basico!A4:A13,0))</f>
+        <v>31000</v>
+      </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -1119,7 +1131,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5A11829-0400-4719-AE5D-0021641EBF77}">
   <dimension ref="A1:J29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
@@ -1165,14 +1177,14 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -1633,7 +1645,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77B0DB54-5707-4E68-9814-271DFFD60495}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.21875" bestFit="1" customWidth="1"/>
@@ -1644,12 +1656,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>

</xml_diff>